<commit_message>
Cabin crew allocation fixed 11-01-2025
</commit_message>
<xml_diff>
--- a/media/downloads/inbound_processed.xlsx
+++ b/media/downloads/inbound_processed.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="34">
   <si>
     <t>DATE</t>
   </si>
@@ -34,7 +34,7 @@
     <t>CREW</t>
   </si>
   <si>
-    <t>09-Jan</t>
+    <t>12-Jan</t>
   </si>
   <si>
     <t>05:00</t>
@@ -55,61 +55,67 @@
     <t>14:30</t>
   </si>
   <si>
-    <t>"SARAB-SAFA"</t>
-  </si>
-  <si>
-    <t>"EM6 "</t>
-  </si>
-  <si>
-    <t>"Talal"</t>
-  </si>
-  <si>
-    <t>"Al Qamzi"</t>
-  </si>
-  <si>
-    <t>"SAB "</t>
-  </si>
-  <si>
-    <t>"FT "</t>
-  </si>
-  <si>
-    <t>"SON "</t>
-  </si>
-  <si>
-    <t>"TECOM "</t>
-  </si>
-  <si>
-    <t>"Dr. K "</t>
-  </si>
-  <si>
-    <t>"MIT "</t>
-  </si>
-  <si>
-    <t>"GCT "</t>
-  </si>
-  <si>
-    <t>"DSO "</t>
-  </si>
-  <si>
-    <t>"MT "</t>
-  </si>
-  <si>
-    <t>"GT"</t>
-  </si>
-  <si>
-    <t>"7Pearls "</t>
-  </si>
-  <si>
-    <t>"PINK "</t>
-  </si>
-  <si>
-    <t>"PZABEEL "</t>
-  </si>
-  <si>
-    <t>"SARAB"</t>
-  </si>
-  <si>
-    <t>"EAC-C"</t>
+    <t>EM6, TALAL, QAMZI</t>
+  </si>
+  <si>
+    <t>SARAB, SAFA</t>
+  </si>
+  <si>
+    <t>SABREEN, FALTAT</t>
+  </si>
+  <si>
+    <t>SONBOULAH</t>
+  </si>
+  <si>
+    <t>TECOM 1,2, DR.KHALIFA</t>
+  </si>
+  <si>
+    <t>MILLINUM TOWER, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>DSO</t>
+  </si>
+  <si>
+    <t>EM6, QAMZI</t>
+  </si>
+  <si>
+    <t>SABREEN, FALTAT, MANAZIL TOWER</t>
+  </si>
+  <si>
+    <t>GARHOUD TOWERS</t>
+  </si>
+  <si>
+    <t>TECOM 1,2</t>
+  </si>
+  <si>
+    <t>7 PEARLS</t>
+  </si>
+  <si>
+    <t>SONBOULAH, GARHOUD TOWERS</t>
+  </si>
+  <si>
+    <t>MILLINUM TOWER, PINK, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>PARK ZABEEL 1,2, 7 PEARLS</t>
+  </si>
+  <si>
+    <t>EM6</t>
+  </si>
+  <si>
+    <t>FALTAT</t>
+  </si>
+  <si>
+    <t>PINK, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>SARAB</t>
+  </si>
+  <si>
+    <t>PARK ZABEEL 1,2</t>
+  </si>
+  <si>
+    <t>EAC-C</t>
   </si>
 </sst>
 </file>
@@ -467,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -504,10 +510,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -524,10 +530,10 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F3">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -544,10 +550,10 @@
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F4">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -564,7 +570,7 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -584,10 +590,10 @@
         <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -604,7 +610,7 @@
         <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -624,7 +630,7 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -638,16 +644,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -658,16 +664,16 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -678,16 +684,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -698,16 +704,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -718,13 +724,13 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F13">
         <v>5</v>
@@ -741,13 +747,13 @@
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F14">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -761,13 +767,13 @@
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F15">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -781,13 +787,13 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -795,19 +801,19 @@
         <v>6</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F17">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -815,19 +821,19 @@
         <v>6</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -838,16 +844,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F19">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -858,16 +864,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20">
         <v>26</v>
-      </c>
-      <c r="E20" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20">
-        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -875,19 +881,19 @@
         <v>6</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F21">
-        <v>5</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -895,19 +901,19 @@
         <v>6</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E22" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -915,19 +921,19 @@
         <v>6</v>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -935,19 +941,19 @@
         <v>6</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E24" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -958,16 +964,16 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E25" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -975,19 +981,19 @@
         <v>6</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F26">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -998,16 +1004,16 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E27" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F27">
-        <v>26</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1018,16 +1024,16 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F28">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1038,16 +1044,16 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F29">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1058,16 +1064,16 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E30" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F30">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1078,16 +1084,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31">
         <v>9</v>
-      </c>
-      <c r="D31" t="s">
-        <v>18</v>
-      </c>
-      <c r="E31" t="s">
-        <v>31</v>
-      </c>
-      <c r="F31">
-        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1098,16 +1104,16 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F32">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1118,16 +1124,16 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F33">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1138,16 +1144,16 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D34" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F34">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1158,16 +1164,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E35" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F35">
-        <v>31</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1178,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F36">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1198,16 +1204,16 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E37" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F37">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1218,16 +1224,16 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D38" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E38" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F38">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1238,16 +1244,16 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D39" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E39" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F39">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1258,16 +1264,16 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E40" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F40">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1275,19 +1281,19 @@
         <v>6</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E41" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F41">
-        <v>59</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1295,19 +1301,19 @@
         <v>6</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D42" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E42" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F42">
-        <v>38</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1318,515 +1324,15 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D43" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E43" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F43">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44" t="s">
-        <v>6</v>
-      </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" t="s">
-        <v>14</v>
-      </c>
-      <c r="E44" t="s">
-        <v>31</v>
-      </c>
-      <c r="F44">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" t="s">
-        <v>6</v>
-      </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" t="s">
-        <v>18</v>
-      </c>
-      <c r="E45" t="s">
-        <v>31</v>
-      </c>
-      <c r="F45">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46" t="s">
-        <v>6</v>
-      </c>
-      <c r="B46">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s">
-        <v>10</v>
-      </c>
-      <c r="D46" t="s">
-        <v>26</v>
-      </c>
-      <c r="E46" t="s">
-        <v>31</v>
-      </c>
-      <c r="F46">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" t="s">
-        <v>20</v>
-      </c>
-      <c r="E47" t="s">
-        <v>31</v>
-      </c>
-      <c r="F47">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48" t="s">
-        <v>6</v>
-      </c>
-      <c r="B48">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s">
-        <v>10</v>
-      </c>
-      <c r="D48" t="s">
-        <v>21</v>
-      </c>
-      <c r="E48" t="s">
-        <v>31</v>
-      </c>
-      <c r="F48">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" t="s">
-        <v>28</v>
-      </c>
-      <c r="E49" t="s">
-        <v>31</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
-      <c r="A50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" t="s">
-        <v>23</v>
-      </c>
-      <c r="E50" t="s">
-        <v>31</v>
-      </c>
-      <c r="F50">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
-      <c r="A51" t="s">
-        <v>6</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" t="s">
-        <v>24</v>
-      </c>
-      <c r="E51" t="s">
-        <v>31</v>
-      </c>
-      <c r="F51">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
-      <c r="A52" t="s">
-        <v>6</v>
-      </c>
-      <c r="B52">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" t="s">
-        <v>14</v>
-      </c>
-      <c r="E52" t="s">
-        <v>31</v>
-      </c>
-      <c r="F52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
-      <c r="A53" t="s">
-        <v>6</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" t="s">
-        <v>15</v>
-      </c>
-      <c r="E53" t="s">
-        <v>31</v>
-      </c>
-      <c r="F53">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
-      <c r="A54" t="s">
-        <v>6</v>
-      </c>
-      <c r="B54">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" t="s">
-        <v>16</v>
-      </c>
-      <c r="E54" t="s">
-        <v>31</v>
-      </c>
-      <c r="F54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
-      <c r="A55" t="s">
-        <v>6</v>
-      </c>
-      <c r="B55">
-        <v>1</v>
-      </c>
-      <c r="C55" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" t="s">
-        <v>30</v>
-      </c>
-      <c r="E55" t="s">
-        <v>31</v>
-      </c>
-      <c r="F55">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
-      <c r="A56" t="s">
-        <v>6</v>
-      </c>
-      <c r="B56">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" t="s">
-        <v>26</v>
-      </c>
-      <c r="E56" t="s">
-        <v>31</v>
-      </c>
-      <c r="F56">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
-      <c r="A57" t="s">
-        <v>6</v>
-      </c>
-      <c r="B57">
-        <v>1</v>
-      </c>
-      <c r="C57" t="s">
-        <v>11</v>
-      </c>
-      <c r="D57" t="s">
-        <v>20</v>
-      </c>
-      <c r="E57" t="s">
-        <v>31</v>
-      </c>
-      <c r="F57">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
-      <c r="A58" t="s">
-        <v>6</v>
-      </c>
-      <c r="B58">
-        <v>1</v>
-      </c>
-      <c r="C58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" t="s">
-        <v>28</v>
-      </c>
-      <c r="E58" t="s">
-        <v>31</v>
-      </c>
-      <c r="F58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6">
-      <c r="A59" t="s">
-        <v>6</v>
-      </c>
-      <c r="B59">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s">
-        <v>23</v>
-      </c>
-      <c r="E59" t="s">
-        <v>31</v>
-      </c>
-      <c r="F59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6">
-      <c r="A60" t="s">
-        <v>6</v>
-      </c>
-      <c r="B60">
-        <v>1</v>
-      </c>
-      <c r="C60" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" t="s">
-        <v>29</v>
-      </c>
-      <c r="E60" t="s">
-        <v>31</v>
-      </c>
-      <c r="F60">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6">
-      <c r="A61" t="s">
-        <v>6</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>12</v>
-      </c>
-      <c r="D61" t="s">
-        <v>30</v>
-      </c>
-      <c r="E61" t="s">
-        <v>31</v>
-      </c>
-      <c r="F61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6">
-      <c r="A62" t="s">
-        <v>6</v>
-      </c>
-      <c r="B62">
-        <v>1</v>
-      </c>
-      <c r="C62" t="s">
-        <v>12</v>
-      </c>
-      <c r="D62" t="s">
-        <v>18</v>
-      </c>
-      <c r="E62" t="s">
-        <v>31</v>
-      </c>
-      <c r="F62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6">
-      <c r="A63" t="s">
-        <v>6</v>
-      </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="C63" t="s">
-        <v>12</v>
-      </c>
-      <c r="D63" t="s">
-        <v>20</v>
-      </c>
-      <c r="E63" t="s">
-        <v>31</v>
-      </c>
-      <c r="F63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6">
-      <c r="A64" t="s">
-        <v>6</v>
-      </c>
-      <c r="B64">
-        <v>1</v>
-      </c>
-      <c r="C64" t="s">
-        <v>12</v>
-      </c>
-      <c r="D64" t="s">
-        <v>22</v>
-      </c>
-      <c r="E64" t="s">
-        <v>31</v>
-      </c>
-      <c r="F64">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6">
-      <c r="A65" t="s">
-        <v>6</v>
-      </c>
-      <c r="B65">
-        <v>1</v>
-      </c>
-      <c r="C65" t="s">
-        <v>12</v>
-      </c>
-      <c r="D65" t="s">
-        <v>23</v>
-      </c>
-      <c r="E65" t="s">
-        <v>31</v>
-      </c>
-      <c r="F65">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6">
-      <c r="A66" t="s">
-        <v>6</v>
-      </c>
-      <c r="B66">
-        <v>1</v>
-      </c>
-      <c r="C66" t="s">
-        <v>12</v>
-      </c>
-      <c r="D66" t="s">
-        <v>29</v>
-      </c>
-      <c r="E66" t="s">
-        <v>31</v>
-      </c>
-      <c r="F66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6">
-      <c r="A67" t="s">
-        <v>6</v>
-      </c>
-      <c r="B67">
-        <v>3</v>
-      </c>
-      <c r="C67" t="s">
-        <v>12</v>
-      </c>
-      <c r="D67" t="s">
-        <v>27</v>
-      </c>
-      <c r="E67" t="s">
-        <v>31</v>
-      </c>
-      <c r="F67">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
-      <c r="A68" t="s">
-        <v>6</v>
-      </c>
-      <c r="B68">
-        <v>1</v>
-      </c>
-      <c r="C68" t="s">
-        <v>12</v>
-      </c>
-      <c r="D68" t="s">
-        <v>24</v>
-      </c>
-      <c r="E68" t="s">
-        <v>31</v>
-      </c>
-      <c r="F68">
         <v>10</v>
       </c>
     </row>

</xml_diff>